<commit_message>
test: ツールのテストと GitHub Actions（Windows PowerShell 5.1 / 7、Linux）を追加
外部モジュールに依存しないテストランナー（tests/Invoke-Tests.ps1）と、
Search-Excel / Export-ExcelToPdf（-CountOnly）/ Invoke-DesignReview の
テスト 35 件を追加。GitHub Actions で Windows PowerShell 5.1・PowerShell 7
（Windows / Linux）の 3 環境で実行する。

- フィクスチャ（tests/fixtures）は make_fixtures.py で生成（共有文字列・ふりがな・
  mc:Fallback の図形・暗号化／破損ファイル・本物の .xls・最小 PDF・誤りを入れた観点表）
- Excel が無い環境では、Excel を使う機能は「理由付きで失敗すること」を確かめる
- 対話モードはクリップボードと Read-Host を関数で差し替えて確かめる

テストで見つけた改善:
- 同梱の観点表に画面一覧の観点（L01 画面IDの重複・記入漏れ、L02 画面遷移と
  画面一覧の一致）を追加（画面一覧に共通の観点しか当たっていなかった）
- Export-ExcelToPdf の一覧で、Windows 以外では先頭に / が残っていたのを修正

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BwaXbva1qG7woHxahpc3op
</commit_message>
<xml_diff>
--- a/tools/review-checklists/詳細設計レビュー観点.xlsx
+++ b/tools/review-checklists/詳細設計レビュー観点.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'観点表'!$A$1:$H$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'観点表'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1464,8 +1464,84 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>画面一覧</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>画面の一覧に漏れや重複がない</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>画面一覧シートの画面IDに重複がなく、すべての画面に画面名・画面区分・概要が記入されている。</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>*画面一覧*</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>画面一覧</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>画面遷移の遷移元・遷移先が画面一覧と一致している</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>画面遷移シートの遷移元画面ID・遷移先画面IDがすべて画面一覧シートにあり、画面名が画面一覧シートと一致している。</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>*画面一覧*</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H26"/>
+  <autoFilter ref="A1:H28"/>
   <dataValidations count="2">
     <dataValidation sqref="E2:E225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>

</xml_diff>

<commit_message>
test: ツールのテストと GitHub Actions（Windows PowerShell 5.1 / 7、Linux）を追加 (#6)
外部モジュールに依存しないテストランナーとテスト 35 件、GitHub Actions（Windows PowerShell 5.1 / PowerShell 7 Windows・Linux）を追加。

テストで見つけて直したもの:
- Invoke-DesignReview: Windows では AppendLine が CRLF を書くため 1 行ごとに 1 文字多く数えられ、依頼の分割数が Linux より増えていた（8000 文字で 10 → 12 件）。プロンプトの改行を LF にそろえた
- 同梱の観点表に画面一覧の観点（L01・L02）を追加
- Export-ExcelToPdf の一覧で Windows 以外では先頭に / が残っていたのを修正
</commit_message>
<xml_diff>
--- a/tools/review-checklists/詳細設計レビュー観点.xlsx
+++ b/tools/review-checklists/詳細設計レビュー観点.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'観点表'!$A$1:$H$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'観点表'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1464,8 +1464,84 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>画面一覧</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>画面の一覧に漏れや重複がない</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>画面一覧シートの画面IDに重複がなく、すべての画面に画面名・画面区分・概要が記入されている。</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>*画面一覧*</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>画面一覧</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>画面遷移の遷移元・遷移先が画面一覧と一致している</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>画面遷移シートの遷移元画面ID・遷移先画面IDがすべて画面一覧シートにあり、画面名が画面一覧シートと一致している。</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>*画面一覧*</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H26"/>
+  <autoFilter ref="A1:H28"/>
   <dataValidations count="2">
     <dataValidation sqref="E2:E225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>

</xml_diff>